<commit_message>
Implement CORDIS ML pipeline and EDA exploration notebook
</commit_message>
<xml_diff>
--- a/Literature_Survey.xlsx
+++ b/Literature_Survey.xlsx
@@ -1,28 +1,207 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/36e9e8dbf8e7e239/Desktop/PROJECTS/CORDIS/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="18" documentId="6_{E43F519E-2D1F-4C59-B800-B79B62AA64F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A334E907-96BA-4708-91C1-7085E671D54B}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="55">
+  <si>
+    <t>Paper Title</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Algorithm/Method</t>
+  </si>
+  <si>
+    <t>Dataset</t>
+  </si>
+  <si>
+    <t>Accuracy</t>
+  </si>
+  <si>
+    <t>Limitation</t>
+  </si>
+  <si>
+    <t>Predicting Heart Diseases Using Machine Learning and Different Data Classification Techniques</t>
+  </si>
+  <si>
+    <t>XGBoost, SVM, RF, KNN, LR, DT</t>
+  </si>
+  <si>
+    <t>Public + Private Heart Disease Datasets</t>
+  </si>
+  <si>
+    <t>97.57%</t>
+  </si>
+  <si>
+    <t>Performance depends on feature selection and balanced data</t>
+  </si>
+  <si>
+    <t>Heart Disease Prediction Using Novel Ensemble and Blending Based Cardiovascular Disease Detection Networks</t>
+  </si>
+  <si>
+    <t>EnsCVDD-Net, BlCVDD-Net</t>
+  </si>
+  <si>
+    <t>Cardiovascular Disease Dataset</t>
+  </si>
+  <si>
+    <t>91.0%</t>
+  </si>
+  <si>
+    <t>Higher computational complexity and training time</t>
+  </si>
+  <si>
+    <t>A Clinical Data Analysis Based Diagnostic Systems for Heart Disease Prediction Using Ensemble Method</t>
+  </si>
+  <si>
+    <t>Logistic Regression, SVM</t>
+  </si>
+  <si>
+    <t>UCI Heart Disease Dataset</t>
+  </si>
+  <si>
+    <t>LR performed best</t>
+  </si>
+  <si>
+    <t>Limited features and traditional ML methods only</t>
+  </si>
+  <si>
+    <t>HDPF: Heart Disease Prediction Framework Based on Hybrid Classifiers and Genetic Algorithm</t>
+  </si>
+  <si>
+    <t>Hybrid Ensemble + Genetic Algorithm</t>
+  </si>
+  <si>
+    <t>98.18%</t>
+  </si>
+  <si>
+    <t>Increased complexity due to hybrid framework</t>
+  </si>
+  <si>
+    <t>Heart Disease Prediction Using a Hybrid Feature Selection and Ensemble Learning Approach</t>
+  </si>
+  <si>
+    <t>CNN + RF + GA + CSO</t>
+  </si>
+  <si>
+    <t>95.0%</t>
+  </si>
+  <si>
+    <t>Optimization increases computational cost</t>
+  </si>
+  <si>
+    <t>Cardiac Clarity: Harnessing Machine Learning for Accurate Heart Disease Prediction</t>
+  </si>
+  <si>
+    <t>RF, LR, KNN, SVM, XGBoost</t>
+  </si>
+  <si>
+    <t>Mendeley Hospital Dataset</t>
+  </si>
+  <si>
+    <t>98.5%</t>
+  </si>
+  <si>
+    <t>Requires extensive hyperparameter tuning</t>
+  </si>
+  <si>
+    <t>Meta-Ensemble Learning for Heart Disease Prediction: A Stacking-Based Approach With Explainable AI</t>
+  </si>
+  <si>
+    <t>LightGBM, RF, XGBoost, Stacking</t>
+  </si>
+  <si>
+    <t>Heart_2020, Cardio Train, Cleveland-Hungary</t>
+  </si>
+  <si>
+    <t>98.90%</t>
+  </si>
+  <si>
+    <t>Complex ensemble architecture</t>
+  </si>
+  <si>
+    <t>A Robust Heart Disease Prediction System Using Hybrid Deep Neural Networks</t>
+  </si>
+  <si>
+    <t>ANN, CNN, LSTM, CNN-LSTM</t>
+  </si>
+  <si>
+    <t>Cleveland + Multi-source Dataset</t>
+  </si>
+  <si>
+    <t>98.86%</t>
+  </si>
+  <si>
+    <t>Deep learning requires higher resources</t>
+  </si>
+  <si>
+    <t>A Clinical Decision Support System for Heart Disease Prediction Using Deep Learning</t>
+  </si>
+  <si>
+    <t>Dense Neural Network (Keras)</t>
+  </si>
+  <si>
+    <t>Multiple Heart Disease Datasets</t>
+  </si>
+  <si>
+    <t>High accuracy</t>
+  </si>
+  <si>
+    <t>Reduced interpretability</t>
+  </si>
+  <si>
+    <t>Heterogeneous Committee-Based Adaptive Active Learning for Efficient Heart Disease Prediction</t>
+  </si>
+  <si>
+    <t>XGBoost, RF, LR with Active Learning</t>
+  </si>
+  <si>
+    <t>Clinical Heart Disease Dataset</t>
+  </si>
+  <si>
+    <t>96.04%</t>
+  </si>
+  <si>
+    <t>Requires iterative labeling</t>
+  </si>
+  <si>
+    <t>Sl No.</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,8 +228,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +515,272 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="93.54296875" customWidth="1"/>
+    <col min="4" max="4" width="33.6328125" customWidth="1"/>
+    <col min="5" max="5" width="39" customWidth="1"/>
+    <col min="6" max="6" width="17.1796875" customWidth="1"/>
+    <col min="7" max="7" width="53" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="2">
+        <v>2025</v>
+      </c>
+      <c r="D6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="2">
+        <v>2025</v>
+      </c>
+      <c r="D7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s">
+        <v>32</v>
+      </c>
+      <c r="G7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="2">
+        <v>2025</v>
+      </c>
+      <c r="D8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" t="s">
+        <v>42</v>
+      </c>
+      <c r="G9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D10" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" t="s">
+        <v>46</v>
+      </c>
+      <c r="F10" t="s">
+        <v>47</v>
+      </c>
+      <c r="G10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="2">
+        <v>2026</v>
+      </c>
+      <c r="D11" t="s">
+        <v>50</v>
+      </c>
+      <c r="E11" t="s">
+        <v>51</v>
+      </c>
+      <c r="F11" t="s">
+        <v>52</v>
+      </c>
+      <c r="G11" t="s">
+        <v>53</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>